<commit_message>
final ba page commit
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekookuniverse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47FF321-FAF0-2D46-BD07-69567ABD47E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C29E047-0E66-CC42-8217-9B21B6205B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="1200" windowWidth="38400" windowHeight="20980" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2696" uniqueCount="1946">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2752" uniqueCount="1982">
   <si>
     <t>date</t>
   </si>
@@ -6557,10 +6557,118 @@
     <t>HUBLOT</t>
   </si>
   <si>
+    <t>CKJK</t>
+  </si>
+  <si>
     <t>HITEJINRO</t>
   </si>
   <si>
-    <t>media</t>
+    <t>JK</t>
+  </si>
+  <si>
+    <t>https://www.calvinklein.us/en/ckjk</t>
+  </si>
+  <si>
+    <t>brandambassador</t>
+  </si>
+  <si>
+    <t>koo_calvinklein.webp</t>
+  </si>
+  <si>
+    <t>koo_ckjk.webp</t>
+  </si>
+  <si>
+    <t>koo_chanel.webp</t>
+  </si>
+  <si>
+    <t>koo_hublot.webp</t>
+  </si>
+  <si>
+    <t>koo_jk.webp</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=lpvR0gjsolI</t>
+  </si>
+  <si>
+    <t>tae_celine.webp</t>
+  </si>
+  <si>
+    <t>tae_cartier.webp</t>
+  </si>
+  <si>
+    <t>tae_siminvest.webp</t>
+  </si>
+  <si>
+    <t>tae_composecoffee.webp</t>
+  </si>
+  <si>
+    <t>tae_snowpeak.webp</t>
+  </si>
+  <si>
+    <t>tae_tirtir.webp</t>
+  </si>
+  <si>
+    <t>tae_yunth.webp</t>
+  </si>
+  <si>
+    <t>tae_hitejinro.webp</t>
+  </si>
+  <si>
+    <t>PARADISE CITY</t>
+  </si>
+  <si>
+    <t>SEOUL TOURISM ORGANIZATION</t>
+  </si>
+  <si>
+    <t>tae_seoultourismorg.webp</t>
+  </si>
+  <si>
+    <t>tae_cocacola.webp</t>
+  </si>
+  <si>
+    <t>https://tirtir.global/</t>
+  </si>
+  <si>
+    <t>https://www.celine.com/</t>
+  </si>
+  <si>
+    <t>https://www.sto.or.kr/</t>
+  </si>
+  <si>
+    <t>https://www.cartier.com/</t>
+  </si>
+  <si>
+    <t>https://siminvest.id/</t>
+  </si>
+  <si>
+    <t>https://composecoffee.com/</t>
+  </si>
+  <si>
+    <t>https://www.coca-cola.com/kr/ko</t>
+  </si>
+  <si>
+    <t>https://www.snowpeakstore.co.kr/</t>
+  </si>
+  <si>
+    <t>https://yunth.jp/</t>
+  </si>
+  <si>
+    <t>https://www.p-city.com/</t>
+  </si>
+  <si>
+    <t>https://hitejinroamerica.com/</t>
+  </si>
+  <si>
+    <t>https://www.calvinklein.us/</t>
+  </si>
+  <si>
+    <t>https://www.chanel.com/</t>
+  </si>
+  <si>
+    <t>https://www.hublot.com/</t>
+  </si>
+  <si>
+    <t>tae_paradisecity.webp</t>
   </si>
 </sst>
 </file>
@@ -57811,11 +57919,13 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64C35039-B9B3-DA4C-95BA-F339368624DF}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -57829,10 +57939,10 @@
         <v>213</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>1945</v>
+        <v>150</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>149</v>
+        <v>434</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>1518</v>
@@ -57845,6 +57955,18 @@
       <c r="B2" t="s">
         <v>1933</v>
       </c>
+      <c r="C2" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1955</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1968</v>
+      </c>
+      <c r="F2">
+        <v>2023</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -57853,6 +57975,18 @@
       <c r="B3" t="s">
         <v>1934</v>
       </c>
+      <c r="C3" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1956</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1970</v>
+      </c>
+      <c r="F3">
+        <v>2023</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -57861,6 +57995,18 @@
       <c r="B4" t="s">
         <v>1935</v>
       </c>
+      <c r="C4" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1957</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>1971</v>
+      </c>
+      <c r="F4">
+        <v>2023</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -57869,6 +58015,18 @@
       <c r="B5" t="s">
         <v>1936</v>
       </c>
+      <c r="C5" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1958</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1972</v>
+      </c>
+      <c r="F5">
+        <v>2023</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -57877,6 +58035,18 @@
       <c r="B6" t="s">
         <v>1937</v>
       </c>
+      <c r="C6" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1966</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1973</v>
+      </c>
+      <c r="F6">
+        <v>2025</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -57885,6 +58055,18 @@
       <c r="B7" t="s">
         <v>1938</v>
       </c>
+      <c r="C7" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1959</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1974</v>
+      </c>
+      <c r="F7">
+        <v>2025</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -57893,6 +58075,18 @@
       <c r="B8" t="s">
         <v>1939</v>
       </c>
+      <c r="C8" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1960</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1967</v>
+      </c>
+      <c r="F8">
+        <v>2025</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -57901,29 +58095,77 @@
       <c r="B9" t="s">
         <v>1940</v>
       </c>
+      <c r="C9" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1961</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1975</v>
+      </c>
+      <c r="F9">
+        <v>2025</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>231</v>
       </c>
       <c r="B10" t="s">
-        <v>1944</v>
+        <v>1963</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1981</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1976</v>
+      </c>
+      <c r="F10">
+        <v>2025</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B11" t="s">
-        <v>1941</v>
+        <v>1945</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1962</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1977</v>
+      </c>
+      <c r="F11">
+        <v>2026</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B12" t="s">
-        <v>1942</v>
+        <v>1964</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1965</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1969</v>
+      </c>
+      <c r="F12">
+        <v>2023</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -57931,10 +58173,109 @@
         <v>221</v>
       </c>
       <c r="B13" t="s">
+        <v>1946</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1953</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>1954</v>
+      </c>
+      <c r="F13">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1941</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1949</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>1978</v>
+      </c>
+      <c r="F14">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>221</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1944</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1950</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>1947</v>
+      </c>
+      <c r="F15">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>221</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1942</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1951</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>1979</v>
+      </c>
+      <c r="F16">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>221</v>
+      </c>
+      <c r="B17" t="s">
         <v>1943</v>
       </c>
+      <c r="C17" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1952</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>1980</v>
+      </c>
+      <c r="F17">
+        <v>2026</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1" display="https://www.youtube.com/watch?v=0thKCJ5Pu0k&amp;t=17s" xr:uid="{41A5E872-AB16-E745-ABB7-8F73E063B69E}"/>
+    <hyperlink ref="E13" r:id="rId2" xr:uid="{BA4B1370-36D3-3A48-A4DB-1C33D850E51A}"/>
+    <hyperlink ref="E14" r:id="rId3" xr:uid="{374FF3EB-AAC2-E44C-85A5-12CD5800A2FB}"/>
+    <hyperlink ref="E16" r:id="rId4" xr:uid="{5AAE3747-957D-3845-989F-707851F55413}"/>
+    <hyperlink ref="E17" r:id="rId5" xr:uid="{EBA670F1-9C27-C94F-8055-EECE2FA9BAA1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
moved recap to main
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekookuniverse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C39F6E2-9A35-BA4B-9F65-56BEB0442282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C99AA1-45FA-A34E-B243-BC5D56F6E316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1180" windowWidth="29560" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="1180" windowWidth="29560" windowHeight="21000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TKURadio" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="1947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2715" uniqueCount="1949">
   <si>
     <t>date</t>
   </si>
@@ -6585,6 +6585,13 @@
   </si>
   <si>
     <t>donations</t>
+  </si>
+  <si>
+    <t>Munich. Paris. More unforgettable moments. 💜💚
+From two incredible concerts in Munich and an unforgettable night in Paris to more content celebrating Taehyung and Jungkook’s work with the brands they represent, plus some of the sweetest personal moments they’ve chosen to share with us, this week gave us so much to celebrate.</t>
+  </si>
+  <si>
+    <t>Week of July 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -61267,7 +61274,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
@@ -61295,13 +61302,13 @@
     </row>
     <row r="2" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="B2" t="s">
-        <v>1942</v>
+        <v>1948</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>1943</v>
+        <v>1947</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>1941</v>
@@ -61310,824 +61317,840 @@
     </row>
     <row r="3" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="B3" t="s">
-        <v>1889</v>
+        <v>1942</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>1891</v>
+        <v>1943</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1890</v>
+        <v>1941</v>
       </c>
       <c r="G3" s="5"/>
     </row>
     <row r="4" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
-        <v>46199</v>
+        <v>46206</v>
       </c>
       <c r="B4" t="s">
-        <v>1770</v>
+        <v>1889</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>1769</v>
+        <v>1891</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1771</v>
+        <v>1890</v>
       </c>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
-        <v>46192</v>
+        <v>46199</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>1770</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>5</v>
+        <v>1769</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>6</v>
+        <v>1771</v>
       </c>
       <c r="G5" s="5"/>
     </row>
     <row r="6" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
-        <v>46185</v>
+        <v>46192</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
-        <v>46171</v>
+        <v>46178</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
-        <v>46164</v>
+        <v>46171</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
-        <v>46157</v>
+        <v>46164</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
-        <v>46143</v>
+        <v>46150</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G12" s="5"/>
     </row>
     <row r="13" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
-        <v>46136</v>
+        <v>46143</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
-        <v>46129</v>
+        <v>46136</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
-        <v>46115</v>
+        <v>46129</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
-        <v>46094</v>
+        <v>46115</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G16" s="5"/>
     </row>
     <row r="17" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
-        <v>46087</v>
+        <v>46094</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G17" s="5"/>
     </row>
     <row r="18" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
-        <v>46080</v>
+        <v>46087</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G18" s="5"/>
     </row>
     <row r="19" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
-        <v>46073</v>
+        <v>46080</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
-        <v>46066</v>
+        <v>46073</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G20" s="5"/>
     </row>
     <row r="21" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
-        <v>46059</v>
+        <v>46066</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>50</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
-        <v>46052</v>
+        <v>46059</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G22" s="5"/>
     </row>
     <row r="23" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
+        <v>46045</v>
+      </c>
+      <c r="B24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G24" s="5"/>
+    </row>
+    <row r="25" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9">
         <v>46038</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C25" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="G24" s="5"/>
-    </row>
-    <row r="25" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="9">
-        <v>46031</v>
-      </c>
-      <c r="B25" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
+        <v>46031</v>
+      </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" s="5"/>
+    </row>
+    <row r="27" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="9">
         <v>46024</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C27" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="G26" s="5"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="9">
-        <v>46017</v>
-      </c>
-      <c r="B27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C27" t="s">
-        <v>69</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="G27" s="5"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
+        <v>46017</v>
+      </c>
+      <c r="B28" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="9">
         <v>46010</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>71</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>72</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="G28" s="5"/>
-    </row>
-    <row r="29" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="9">
-        <v>46003</v>
-      </c>
-      <c r="B29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="G29" s="5"/>
     </row>
     <row r="30" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
-        <v>45996</v>
+        <v>46003</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="G30" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
-        <v>45989</v>
+        <v>45996</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G31" s="6"/>
     </row>
     <row r="32" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
-        <v>45982</v>
+        <v>45989</v>
       </c>
       <c r="B32" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G32" s="6"/>
     </row>
     <row r="33" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
-        <v>45975</v>
+        <v>45982</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
-        <v>45968</v>
+        <v>45975</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
+        <v>45968</v>
+      </c>
+      <c r="B35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="9">
         <v>45961</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>90</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C36" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D36" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G35" s="6"/>
-    </row>
-    <row r="36" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="9">
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="9">
         <v>45954</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>93</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C37" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D37" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G36" s="6"/>
-    </row>
-    <row r="37" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="9">
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="9">
         <v>45947</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C38" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D38" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="9">
+      <c r="G38" s="6"/>
+    </row>
+    <row r="39" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="9">
         <v>45940</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>99</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C39" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D39" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="39" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="9">
-        <v>45933</v>
-      </c>
-      <c r="B39" t="s">
-        <v>102</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="G39" s="6"/>
     </row>
     <row r="40" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
+        <v>45933</v>
+      </c>
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="9">
         <v>45926</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>105</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C41" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D41" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="G40" s="6"/>
-    </row>
-    <row r="41" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="9">
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="9">
         <v>45919</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>108</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C42" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D42" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="9">
-        <v>45912</v>
-      </c>
-      <c r="B42" t="s">
-        <v>111</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="G42" s="6"/>
     </row>
     <row r="43" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
+        <v>45912</v>
+      </c>
+      <c r="B43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G43" s="6"/>
+    </row>
+    <row r="44" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="9">
         <v>45905</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C44" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D44" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="9">
+      <c r="G44" s="6"/>
+    </row>
+    <row r="45" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="9">
         <v>45898</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>117</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C45" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D45" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="G44" s="6"/>
-    </row>
-    <row r="45" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="9">
+      <c r="G45" s="6"/>
+    </row>
+    <row r="46" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="9">
         <v>45891</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>120</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C46" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D46" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="9">
+      <c r="G46" s="6"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="9">
         <v>45884</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>123</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>123</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D47" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="9">
-        <v>45877</v>
-      </c>
-      <c r="B47" t="s">
-        <v>125</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="G47" s="6"/>
     </row>
     <row r="48" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
+        <v>45877</v>
+      </c>
+      <c r="B48" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G48" s="6"/>
+    </row>
+    <row r="49" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="9">
         <v>45870</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C49" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D49" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="G48" s="6"/>
-    </row>
-    <row r="49" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="9">
-        <v>45863</v>
-      </c>
-      <c r="B49" t="s">
-        <v>131</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9">
-        <v>45856</v>
+        <v>45863</v>
       </c>
       <c r="B50" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G50" s="6"/>
     </row>
     <row r="51" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9">
-        <v>45849</v>
+        <v>45856</v>
       </c>
       <c r="B51" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G51" s="6"/>
     </row>
     <row r="52" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G52" s="6"/>
     </row>
     <row r="53" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="9">
+        <v>45842</v>
+      </c>
+      <c r="B53" t="s">
+        <v>140</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G53" s="6"/>
+    </row>
+    <row r="54" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="9">
         <v>45835</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>143</v>
       </c>
-      <c r="C53" s="8" t="s">
+      <c r="C54" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D54" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="G53" s="6"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="C54" s="8"/>
+      <c r="G54" s="6"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C55" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="D6" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="D7" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
-    <hyperlink ref="D8" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
-    <hyperlink ref="D9" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
-    <hyperlink ref="D10" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
-    <hyperlink ref="D11" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
-    <hyperlink ref="D13" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
-    <hyperlink ref="D15" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
-    <hyperlink ref="D16" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
-    <hyperlink ref="D17" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
-    <hyperlink ref="D18" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
-    <hyperlink ref="D19" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
-    <hyperlink ref="D20" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
-    <hyperlink ref="D21" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
-    <hyperlink ref="D22" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
-    <hyperlink ref="D23" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
-    <hyperlink ref="D24" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
-    <hyperlink ref="D25" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
-    <hyperlink ref="D26" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
-    <hyperlink ref="D27" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
-    <hyperlink ref="D28" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
-    <hyperlink ref="D29" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
-    <hyperlink ref="D30" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
-    <hyperlink ref="D31" r:id="rId25" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
-    <hyperlink ref="D32" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
-    <hyperlink ref="D33" r:id="rId27" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
-    <hyperlink ref="D34" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
-    <hyperlink ref="D35" r:id="rId29" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
-    <hyperlink ref="D36" r:id="rId30" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
-    <hyperlink ref="D37" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
-    <hyperlink ref="D38" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
-    <hyperlink ref="D39" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
-    <hyperlink ref="D40" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
-    <hyperlink ref="D41" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
-    <hyperlink ref="D42" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
-    <hyperlink ref="D43" r:id="rId37" xr:uid="{00000000-0004-0000-0400-000024000000}"/>
-    <hyperlink ref="D44" r:id="rId38" xr:uid="{00000000-0004-0000-0400-000025000000}"/>
-    <hyperlink ref="D45" r:id="rId39" xr:uid="{00000000-0004-0000-0400-000026000000}"/>
-    <hyperlink ref="D46" r:id="rId40" xr:uid="{00000000-0004-0000-0400-000027000000}"/>
-    <hyperlink ref="D47" r:id="rId41" xr:uid="{00000000-0004-0000-0400-000028000000}"/>
-    <hyperlink ref="D48" r:id="rId42" xr:uid="{00000000-0004-0000-0400-000029000000}"/>
-    <hyperlink ref="D49" r:id="rId43" xr:uid="{00000000-0004-0000-0400-00002A000000}"/>
-    <hyperlink ref="D50" r:id="rId44" xr:uid="{00000000-0004-0000-0400-00002B000000}"/>
-    <hyperlink ref="D51" r:id="rId45" xr:uid="{00000000-0004-0000-0400-00002C000000}"/>
-    <hyperlink ref="D52" r:id="rId46" xr:uid="{00000000-0004-0000-0400-00002D000000}"/>
-    <hyperlink ref="D53" r:id="rId47" xr:uid="{00000000-0004-0000-0400-00002E000000}"/>
-    <hyperlink ref="D5" r:id="rId48" xr:uid="{F9990143-F9A9-124E-BCC1-1FAB349A9366}"/>
-    <hyperlink ref="D4" r:id="rId49" xr:uid="{EE336F4B-5EFC-034A-9FF6-DB34FC42BBA7}"/>
-    <hyperlink ref="D3" r:id="rId50" xr:uid="{4FE02816-5803-B546-8B3C-00FB300D94B2}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="D8" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="D9" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="D10" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="D11" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="D12" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="D14" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="D16" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="D17" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="D18" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="D19" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="D20" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="D21" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="D22" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="D23" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="D24" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="D25" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
+    <hyperlink ref="D26" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
+    <hyperlink ref="D27" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
+    <hyperlink ref="D28" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
+    <hyperlink ref="D29" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
+    <hyperlink ref="D30" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
+    <hyperlink ref="D31" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
+    <hyperlink ref="D32" r:id="rId25" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
+    <hyperlink ref="D33" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
+    <hyperlink ref="D34" r:id="rId27" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
+    <hyperlink ref="D35" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
+    <hyperlink ref="D36" r:id="rId29" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
+    <hyperlink ref="D37" r:id="rId30" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
+    <hyperlink ref="D38" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
+    <hyperlink ref="D39" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
+    <hyperlink ref="D40" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
+    <hyperlink ref="D41" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
+    <hyperlink ref="D42" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
+    <hyperlink ref="D43" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
+    <hyperlink ref="D44" r:id="rId37" xr:uid="{00000000-0004-0000-0400-000024000000}"/>
+    <hyperlink ref="D45" r:id="rId38" xr:uid="{00000000-0004-0000-0400-000025000000}"/>
+    <hyperlink ref="D46" r:id="rId39" xr:uid="{00000000-0004-0000-0400-000026000000}"/>
+    <hyperlink ref="D47" r:id="rId40" xr:uid="{00000000-0004-0000-0400-000027000000}"/>
+    <hyperlink ref="D48" r:id="rId41" xr:uid="{00000000-0004-0000-0400-000028000000}"/>
+    <hyperlink ref="D49" r:id="rId42" xr:uid="{00000000-0004-0000-0400-000029000000}"/>
+    <hyperlink ref="D50" r:id="rId43" xr:uid="{00000000-0004-0000-0400-00002A000000}"/>
+    <hyperlink ref="D51" r:id="rId44" xr:uid="{00000000-0004-0000-0400-00002B000000}"/>
+    <hyperlink ref="D52" r:id="rId45" xr:uid="{00000000-0004-0000-0400-00002C000000}"/>
+    <hyperlink ref="D53" r:id="rId46" xr:uid="{00000000-0004-0000-0400-00002D000000}"/>
+    <hyperlink ref="D54" r:id="rId47" xr:uid="{00000000-0004-0000-0400-00002E000000}"/>
+    <hyperlink ref="D6" r:id="rId48" xr:uid="{F9990143-F9A9-124E-BCC1-1FAB349A9366}"/>
+    <hyperlink ref="D5" r:id="rId49" xr:uid="{EE336F4B-5EFC-034A-9FF6-DB34FC42BBA7}"/>
+    <hyperlink ref="D4" r:id="rId50" xr:uid="{4FE02816-5803-B546-8B3C-00FB300D94B2}"/>
+    <hyperlink ref="D3" r:id="rId51" xr:uid="{8E240BDD-02FF-CA47-B5D9-FD7E9FCA5AEA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added who said it
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekookuniverse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5271CD62-649B-1943-ABF7-2AA4D1A2CB74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{445D6E5B-3311-2945-8044-FB5DCC1D69ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1180" windowWidth="29560" windowHeight="21000" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="1360" windowWidth="29560" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TKURadio" sheetId="1" r:id="rId1"/>
@@ -60752,9 +60752,7 @@
       <c r="F9" t="s">
         <v>176</v>
       </c>
-      <c r="P9" s="27">
-        <v>1137205471</v>
-      </c>
+      <c r="P9" s="27"/>
     </row>
     <row r="10" spans="1:16" ht="18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -60766,9 +60764,7 @@
       <c r="F10" t="s">
         <v>172</v>
       </c>
-      <c r="P10" s="27">
-        <v>379548571</v>
-      </c>
+      <c r="P10" s="27"/>
     </row>
     <row r="11" spans="1:16" ht="18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -60780,9 +60776,7 @@
       <c r="F11" t="s">
         <v>176</v>
       </c>
-      <c r="P11" s="28">
-        <v>172090822</v>
-      </c>
+      <c r="P11" s="28"/>
     </row>
     <row r="12" spans="1:16" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -60794,9 +60788,7 @@
       <c r="F12" t="s">
         <v>168</v>
       </c>
-      <c r="P12" s="27">
-        <v>585285626</v>
-      </c>
+      <c r="P12" s="27"/>
     </row>
     <row r="13" spans="1:16" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -60808,9 +60800,7 @@
       <c r="F13" t="s">
         <v>176</v>
       </c>
-      <c r="P13" s="27">
-        <v>178700934</v>
-      </c>
+      <c r="P13" s="27"/>
     </row>
     <row r="14" spans="1:16" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -60822,9 +60812,7 @@
       <c r="F14" t="s">
         <v>172</v>
       </c>
-      <c r="P14" s="27">
-        <v>147468974</v>
-      </c>
+      <c r="P14" s="27"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -60836,10 +60824,7 @@
       <c r="F15" t="s">
         <v>168</v>
       </c>
-      <c r="P15" s="26">
-        <f>SUM(P9:P14)</f>
-        <v>2600300398</v>
-      </c>
+      <c r="P15" s="26"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">

</xml_diff>

<commit_message>
Doenjang Curry Pasta update
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekookuniverse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C524A6-9005-DC47-9396-6D0CF9F31B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EF5D34-B49C-BB42-A21F-49901975B1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31520" yWindow="1180" windowWidth="29560" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-31520" yWindow="1180" windowWidth="29560" windowHeight="21000" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TKURadio" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3924" uniqueCount="2473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3940" uniqueCount="2485">
   <si>
     <t>date</t>
   </si>
@@ -12590,9 +12590,6 @@
     <t>https://weverse.io/bts/live/3-215169045</t>
   </si>
   <si>
-    <t>media</t>
-  </si>
-  <si>
     <t>playlist_group</t>
   </si>
   <si>
@@ -12873,6 +12870,106 @@
   </si>
   <si>
     <t>Winter_Ahead_with_PARK_HYO_SHIN_YUNSEOKCHEOL_TRIO_.webp</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rJqlnCywaBc</t>
+  </si>
+  <si>
+    <t>Week of August 1, 2026</t>
+  </si>
+  <si>
+    <t>Even without a concert, Taehyung and Jungkook still gave us tons of content to enjoy and celebrate. From brand content, behind-the-scenes moments from the “Normal” MV shoot, to personal updates and JK Live, twice, we had another full week!💜</t>
+  </si>
+  <si>
+    <t>Doenjang Curry Pasta</t>
+  </si>
+  <si>
+    <t>35 min</t>
+  </si>
+  <si>
+    <t>doenjang_curry_pasta.png</t>
+  </si>
+  <si>
+    <t>During his December 3, 2025 Weverse Live, Jungkook experimented with creating a completely original pasta recipe using doenjang and Golden Curry. Although he enjoyed the finished dish, he concluded that the flavorful sauce paired even better with rice, showcasing his love for comforting home-style meals and playful experimentation in the kitchen.</t>
+  </si>
+  <si>
+    <t>video</t>
+  </si>
+  <si>
+    <t>Bring a pot of salted water to a boil and cook the pasta until al dente (about 8–10 minutes). Reserve some pasta water before draining.
+Dice the potato into very small cubes. Thinly slice the bacon. Julienne the onion.
+Heat olive oil over low heat and slowly sauté the bacon until lightly crisp.
+Transfer the bacon and its flavorful oil to a plate.
+Add butter (or a little more olive oil) to the pan.
+Add the onion and sauté until softened.
+Stir in the diced potatoes.
+Season with salt and black pepper.
+Cook until the potatoes begin to soften.
+Add ½ teaspoon doenjang (soybean paste) and stir until dissolved.
+Return about half of the cooked bacon together with its reserved oil.
+Pour in a splash of water.
+Add ½ teaspoon Golden Curry and stir until fully dissolved.
+Add a pinch of sugar.
+Stir in 1 tablespoon heavy cream.
+Add more water if the sauce becomes too thick.
+Bring everything to a gentle simmer.
+Add the cooked pasta.
+Add a little pasta water if needed and toss everything together.
+Cook for about 3 minutes, allowing the sauce to fully coat the noodles.
+Add red pepper flakes to taste.
+Stir in chopped parsley.
+Jungkook added about 3 more spoonfuls of water before performing mantecare—vigorously tossing the pasta until the sauce became smooth and glossy.
+Plate the pasta.
+Top with the remaining bacon and garnish with more parsley and red pepper flakes.</t>
+  </si>
+  <si>
+    <t>This was one of Jungkook's own original recipe tryouts, and throughout the live, he was skeptical about how the dish would turn out. His childhood friend from Busan was with him, and Jungkook joked that if the pasta turned out badly, they would simply order delivery afterward.
+While the curry was almost ready, he showed us the output and specified that the color looked like Danhobak-juk (Sweet Pumpkin Porridge) because of its warm golden-orange color. 
+He also mentioned several times that the sauce would probably be delicious with udon noodles.
+While eating, he said that he could have done Risotto with it. He even asked his house helper ("Emo"—a respectful Korean term meaning "Auntie") for a bowl of cooked rice, mixed it into the remaining sauce, and happily ate it. After trying it with rice, he felt the sauce actually paired better with rice than pasta.</t>
+  </si>
+  <si>
+    <t>Pasta (about 200 g)*
+1 potato, finely diced
+1 onion, julienned
+Bacon (quantity not specified)
+Olive oil (amount not specified)
+Butter (amount not specified)
+Doenjang (about ½ tsp)*
+Golden Curry (about ½ cube)*
+Heavy cream (about 1 tbsp)*
+Sugar (a pinch, as shown)
+Salt
+Black pepper
+Water
+Pasta water
+Red pepper flakes
+Parsley</t>
+  </si>
+  <si>
+    <t>A rich and creamy fusion pasta created by Jungkook, combining Korean doenjang with Japanese Golden Curry for a unique blend of savory, umami flavors.</t>
+  </si>
+  <si>
+    <t>Dice the potatoes very small so they soften quickly and naturally thicken the sauce.
+Finely sliced onions release moisture faster and develop more sweetness.
+The starch from the potatoes creates a naturally creamy texture.
+Because both doenjang and curry already contain salt, Jungkook intentionally used less pasta water than he normally would.
+The recipe also works well with udon noodles.
+The sauce can easily be transformed into a risotto by stirring cooked rice into it.
+In Korea, it's common to mix leftover rice into a flavorful soup or sauce (국물, gukmul) after finishing the noodles.
+*Estimated measurements are based on observing the livestream.
+---
+🌏 Cultural Notes
+Doenjang (된장)
+Traditional Korean fermented soybean paste with a deep, salty, umami flavor.
+Golden Curry
+A Japanese curry roux commonly sold in cube form.
+Danhobak-juk (단호박죽)
+Korean sweet pumpkin porridge.
+Mantecare
+An Italian cooking technique of vigorously tossing pasta with sauce to create a smooth, emulsified texture.
+Jjigae (찌개)
+A Korean stew, such as kimchi-jjigae.</t>
   </si>
 </sst>
 </file>
@@ -13419,10 +13516,10 @@
         <v>2193</v>
       </c>
       <c r="G1" t="s">
+        <v>2378</v>
+      </c>
+      <c r="H1" t="s">
         <v>2379</v>
-      </c>
-      <c r="H1" t="s">
-        <v>2380</v>
       </c>
       <c r="I1" t="s">
         <v>2194</v>
@@ -13454,7 +13551,7 @@
         <v>2063</v>
       </c>
       <c r="G2" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H2" t="s">
         <v>2178</v>
@@ -13471,7 +13568,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2381</v>
+        <v>2380</v>
       </c>
       <c r="C3" t="s">
         <v>2179</v>
@@ -13486,10 +13583,10 @@
         <v>2063</v>
       </c>
       <c r="G3" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="H3" t="s">
-        <v>2382</v>
+        <v>2381</v>
       </c>
       <c r="I3" t="s">
         <v>512</v>
@@ -13503,7 +13600,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>2383</v>
+        <v>2382</v>
       </c>
       <c r="C4" t="s">
         <v>2181</v>
@@ -13518,7 +13615,7 @@
         <v>2063</v>
       </c>
       <c r="G4" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="H4" t="s">
         <v>2195</v>
@@ -13535,7 +13632,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>2384</v>
+        <v>2383</v>
       </c>
       <c r="C5" t="s">
         <v>2183</v>
@@ -13550,7 +13647,7 @@
         <v>2185</v>
       </c>
       <c r="G5" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H5" t="s">
         <v>2186</v>
@@ -13585,7 +13682,7 @@
         <v>2185</v>
       </c>
       <c r="G6" t="s">
-        <v>2447</v>
+        <v>2446</v>
       </c>
       <c r="H6" t="s">
         <v>2189</v>
@@ -13602,7 +13699,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>2385</v>
+        <v>2384</v>
       </c>
       <c r="C7" t="s">
         <v>2196</v>
@@ -13617,7 +13714,7 @@
         <v>2185</v>
       </c>
       <c r="G7" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H7" t="s">
         <v>2198</v>
@@ -13629,7 +13726,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>2386</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -13637,7 +13734,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>2387</v>
+        <v>2386</v>
       </c>
       <c r="C8" t="s">
         <v>2199</v>
@@ -13652,7 +13749,7 @@
         <v>2185</v>
       </c>
       <c r="G8" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H8" t="s">
         <v>2198</v>
@@ -13664,7 +13761,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>2388</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -13687,7 +13784,7 @@
         <v>2185</v>
       </c>
       <c r="G9" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H9" t="s">
         <v>2203</v>
@@ -13719,7 +13816,7 @@
         <v>2185</v>
       </c>
       <c r="G10" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H10" t="s">
         <v>2206</v>
@@ -13751,7 +13848,7 @@
         <v>2185</v>
       </c>
       <c r="G11" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H11" t="s">
         <v>2186</v>
@@ -13763,7 +13860,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>2389</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
@@ -13786,7 +13883,7 @@
         <v>2185</v>
       </c>
       <c r="G12" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H12" t="s">
         <v>2186</v>
@@ -13798,7 +13895,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="s">
-        <v>2390</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -13821,7 +13918,7 @@
         <v>2063</v>
       </c>
       <c r="G13" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H13" t="s">
         <v>2213</v>
@@ -13853,7 +13950,7 @@
         <v>2063</v>
       </c>
       <c r="G14" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H14" t="s">
         <v>2178</v>
@@ -13885,7 +13982,7 @@
         <v>2063</v>
       </c>
       <c r="G15" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="H15" t="s">
         <v>2218</v>
@@ -13902,7 +13999,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>2391</v>
+        <v>2390</v>
       </c>
       <c r="C16" t="s">
         <v>2219</v>
@@ -13914,10 +14011,10 @@
         <v>423</v>
       </c>
       <c r="F16" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G16" t="s">
-        <v>2447</v>
+        <v>2446</v>
       </c>
       <c r="H16" t="s">
         <v>2189</v>
@@ -13934,7 +14031,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>2393</v>
+        <v>2392</v>
       </c>
       <c r="C17" t="s">
         <v>2221</v>
@@ -13946,10 +14043,10 @@
         <v>423</v>
       </c>
       <c r="F17" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G17" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H17" t="s">
         <v>2186</v>
@@ -13961,7 +14058,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>2394</v>
+        <v>2393</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -13969,7 +14066,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>2395</v>
+        <v>2394</v>
       </c>
       <c r="C18" t="s">
         <v>2223</v>
@@ -13981,10 +14078,10 @@
         <v>423</v>
       </c>
       <c r="F18" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G18" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H18" t="s">
         <v>2186</v>
@@ -13996,7 +14093,7 @@
         <v>1</v>
       </c>
       <c r="K18" t="s">
-        <v>2396</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -14004,7 +14101,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>2397</v>
+        <v>2396</v>
       </c>
       <c r="C19" t="s">
         <v>2223</v>
@@ -14016,10 +14113,10 @@
         <v>423</v>
       </c>
       <c r="F19" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G19" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H19" t="s">
         <v>2186</v>
@@ -14031,7 +14128,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="s">
-        <v>2398</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -14039,7 +14136,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>2399</v>
+        <v>2398</v>
       </c>
       <c r="C20" t="s">
         <v>2225</v>
@@ -14051,10 +14148,10 @@
         <v>423</v>
       </c>
       <c r="F20" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G20" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H20" t="s">
         <v>2227</v>
@@ -14071,7 +14168,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>2400</v>
+        <v>2399</v>
       </c>
       <c r="C21" t="s">
         <v>2228</v>
@@ -14083,10 +14180,10 @@
         <v>423</v>
       </c>
       <c r="F21" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G21" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H21" t="s">
         <v>2186</v>
@@ -14098,7 +14195,7 @@
         <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>2401</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -14106,7 +14203,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>2402</v>
+        <v>2401</v>
       </c>
       <c r="C22" t="s">
         <v>2228</v>
@@ -14118,10 +14215,10 @@
         <v>423</v>
       </c>
       <c r="F22" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G22" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H22" t="s">
         <v>2230</v>
@@ -14150,10 +14247,10 @@
         <v>423</v>
       </c>
       <c r="F23" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G23" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H23" t="s">
         <v>2186</v>
@@ -14165,7 +14262,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>2403</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
@@ -14173,7 +14270,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>2404</v>
+        <v>2403</v>
       </c>
       <c r="C24" t="s">
         <v>2233</v>
@@ -14185,10 +14282,10 @@
         <v>423</v>
       </c>
       <c r="F24" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="G24" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H24" t="s">
         <v>2235</v>
@@ -14200,7 +14297,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="s">
-        <v>2405</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -14223,7 +14320,7 @@
         <v>2063</v>
       </c>
       <c r="G25" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H25" t="s">
         <v>2178</v>
@@ -14240,7 +14337,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>2406</v>
+        <v>2405</v>
       </c>
       <c r="C26" t="s">
         <v>2238</v>
@@ -14255,7 +14352,7 @@
         <v>2063</v>
       </c>
       <c r="G26" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="H26" t="s">
         <v>2195</v>
@@ -14284,10 +14381,10 @@
         <v>423</v>
       </c>
       <c r="F27" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G27" t="s">
-        <v>2447</v>
+        <v>2446</v>
       </c>
       <c r="H27" t="s">
         <v>2189</v>
@@ -14316,10 +14413,10 @@
         <v>423</v>
       </c>
       <c r="F28" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G28" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H28" t="s">
         <v>2186</v>
@@ -14331,7 +14428,7 @@
         <v>1</v>
       </c>
       <c r="K28" t="s">
-        <v>2408</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -14351,10 +14448,10 @@
         <v>423</v>
       </c>
       <c r="F29" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G29" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H29" t="s">
         <v>2186</v>
@@ -14366,7 +14463,7 @@
         <v>1</v>
       </c>
       <c r="K29" t="s">
-        <v>2409</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -14386,10 +14483,10 @@
         <v>423</v>
       </c>
       <c r="F30" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G30" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H30" t="s">
         <v>2186</v>
@@ -14401,7 +14498,7 @@
         <v>1</v>
       </c>
       <c r="K30" t="s">
-        <v>2410</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -14421,10 +14518,10 @@
         <v>423</v>
       </c>
       <c r="F31" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G31" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H31" t="s">
         <v>2248</v>
@@ -14436,7 +14533,7 @@
         <v>1</v>
       </c>
       <c r="K31" t="s">
-        <v>2411</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -14456,10 +14553,10 @@
         <v>423</v>
       </c>
       <c r="F32" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G32" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H32" t="s">
         <v>2186</v>
@@ -14471,7 +14568,7 @@
         <v>1</v>
       </c>
       <c r="K32" t="s">
-        <v>2412</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
@@ -14491,10 +14588,10 @@
         <v>423</v>
       </c>
       <c r="F33" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="G33" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="H33" t="s">
         <v>2186</v>
@@ -14506,7 +14603,7 @@
         <v>1</v>
       </c>
       <c r="K33" t="s">
-        <v>2413</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -14529,7 +14626,7 @@
         <v>2063</v>
       </c>
       <c r="G34" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H34" t="s">
         <v>2213</v>
@@ -14561,7 +14658,7 @@
         <v>2063</v>
       </c>
       <c r="G35" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H35" t="s">
         <v>2213</v>
@@ -14593,7 +14690,7 @@
         <v>2063</v>
       </c>
       <c r="G36" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H36" t="s">
         <v>2213</v>
@@ -14625,7 +14722,7 @@
         <v>2063</v>
       </c>
       <c r="G37" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H37" t="s">
         <v>2213</v>
@@ -14657,7 +14754,7 @@
         <v>2063</v>
       </c>
       <c r="G38" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H38" t="s">
         <v>2213</v>
@@ -14689,7 +14786,7 @@
         <v>2063</v>
       </c>
       <c r="G39" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="H39" t="s">
         <v>2213</v>
@@ -14721,7 +14818,7 @@
         <v>618</v>
       </c>
       <c r="G40" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H40" t="s">
         <v>2289</v>
@@ -14753,7 +14850,7 @@
         <v>916</v>
       </c>
       <c r="G41" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H41" t="s">
         <v>2268</v>
@@ -14785,7 +14882,7 @@
         <v>601</v>
       </c>
       <c r="G42" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H42" t="s">
         <v>2268</v>
@@ -14817,7 +14914,7 @@
         <v>743</v>
       </c>
       <c r="G43" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H43" t="s">
         <v>2273</v>
@@ -14849,7 +14946,7 @@
         <v>1028</v>
       </c>
       <c r="G44" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H44" t="s">
         <v>2276</v>
@@ -14881,7 +14978,7 @@
         <v>2279</v>
       </c>
       <c r="G45" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H45" t="s">
         <v>2268</v>
@@ -14913,7 +15010,7 @@
         <v>748</v>
       </c>
       <c r="G46" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H46" t="s">
         <v>2282</v>
@@ -14925,7 +15022,7 @@
         <v>1</v>
       </c>
       <c r="K46" t="s">
-        <v>2414</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
@@ -14948,7 +15045,7 @@
         <v>498</v>
       </c>
       <c r="G47" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H47" t="s">
         <v>2178</v>
@@ -14960,7 +15057,7 @@
         <v>1</v>
       </c>
       <c r="K47" t="s">
-        <v>2415</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -14968,7 +15065,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>2416</v>
+        <v>2415</v>
       </c>
       <c r="C48" t="s">
         <v>2285</v>
@@ -14983,7 +15080,7 @@
         <v>2065</v>
       </c>
       <c r="G48" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H48" t="s">
         <v>2282</v>
@@ -14995,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="K48" t="s">
-        <v>2417</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
@@ -15018,7 +15115,7 @@
         <v>613</v>
       </c>
       <c r="G49" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
       <c r="H49" t="s">
         <v>2289</v>
@@ -15050,7 +15147,7 @@
         <v>757</v>
       </c>
       <c r="G50" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H50" t="s">
         <v>2178</v>
@@ -15067,7 +15164,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>2418</v>
+        <v>2417</v>
       </c>
       <c r="C51" t="s">
         <v>2292</v>
@@ -15082,7 +15179,7 @@
         <v>2069</v>
       </c>
       <c r="G51" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
       <c r="H51" t="s">
         <v>2282</v>
@@ -15094,7 +15191,7 @@
         <v>1</v>
       </c>
       <c r="K51" t="s">
-        <v>2419</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
@@ -15102,7 +15199,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>2420</v>
+        <v>2419</v>
       </c>
       <c r="C52" t="s">
         <v>2294</v>
@@ -15114,10 +15211,10 @@
         <v>421</v>
       </c>
       <c r="F52" t="s">
-        <v>2421</v>
+        <v>2420</v>
       </c>
       <c r="G52" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
       <c r="H52" t="s">
         <v>2186</v>
@@ -15129,7 +15226,7 @@
         <v>1</v>
       </c>
       <c r="K52" t="s">
-        <v>2422</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
@@ -15137,7 +15234,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>2423</v>
+        <v>2422</v>
       </c>
       <c r="C53" t="s">
         <v>2296</v>
@@ -15149,10 +15246,10 @@
         <v>421</v>
       </c>
       <c r="F53" t="s">
-        <v>2421</v>
+        <v>2420</v>
       </c>
       <c r="G53" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
       <c r="H53" t="s">
         <v>2189</v>
@@ -15169,7 +15266,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>2424</v>
+        <v>2423</v>
       </c>
       <c r="C54" t="s">
         <v>2298</v>
@@ -15181,10 +15278,10 @@
         <v>421</v>
       </c>
       <c r="F54" t="s">
-        <v>2421</v>
+        <v>2420</v>
       </c>
       <c r="G54" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
       <c r="H54" t="s">
         <v>2300</v>
@@ -15216,7 +15313,7 @@
         <v>809</v>
       </c>
       <c r="G55" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H55" t="s">
         <v>2178</v>
@@ -15248,7 +15345,7 @@
         <v>809</v>
       </c>
       <c r="G56" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H56" t="s">
         <v>2178</v>
@@ -15280,7 +15377,7 @@
         <v>809</v>
       </c>
       <c r="G57" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H57" t="s">
         <v>2178</v>
@@ -15312,7 +15409,7 @@
         <v>809</v>
       </c>
       <c r="G58" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H58" t="s">
         <v>2178</v>
@@ -15344,7 +15441,7 @@
         <v>809</v>
       </c>
       <c r="G59" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H59" t="s">
         <v>2213</v>
@@ -15361,7 +15458,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>2425</v>
+        <v>2424</v>
       </c>
       <c r="C60" t="s">
         <v>2311</v>
@@ -15376,7 +15473,7 @@
         <v>809</v>
       </c>
       <c r="G60" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="H60" t="s">
         <v>2313</v>
@@ -15408,7 +15505,7 @@
         <v>916</v>
       </c>
       <c r="G61" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H61" t="s">
         <v>2268</v>
@@ -15440,7 +15537,7 @@
         <v>2279</v>
       </c>
       <c r="G62" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H62" t="s">
         <v>2268</v>
@@ -15472,7 +15569,7 @@
         <v>601</v>
       </c>
       <c r="G63" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H63" t="s">
         <v>2268</v>
@@ -15504,7 +15601,7 @@
         <v>2061</v>
       </c>
       <c r="G64" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H64" t="s">
         <v>2276</v>
@@ -15536,7 +15633,7 @@
         <v>2061</v>
       </c>
       <c r="G65" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
       <c r="H65" t="s">
         <v>2189</v>
@@ -15568,7 +15665,7 @@
         <v>2064</v>
       </c>
       <c r="G66" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H66" t="s">
         <v>2327</v>
@@ -15600,7 +15697,7 @@
         <v>2330</v>
       </c>
       <c r="G67" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H67" t="s">
         <v>2276</v>
@@ -15632,7 +15729,7 @@
         <v>2330</v>
       </c>
       <c r="G68" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
       <c r="H68" t="s">
         <v>2189</v>
@@ -15664,7 +15761,7 @@
         <v>922</v>
       </c>
       <c r="G69" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H69" t="s">
         <v>2273</v>
@@ -15696,7 +15793,7 @@
         <v>870</v>
       </c>
       <c r="G70" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="H70" t="s">
         <v>2273</v>
@@ -15728,7 +15825,7 @@
         <v>2340</v>
       </c>
       <c r="G71" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
       <c r="H71" t="s">
         <v>2276</v>
@@ -15740,7 +15837,7 @@
         <v>1</v>
       </c>
       <c r="K71" t="s">
-        <v>2426</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
@@ -15748,7 +15845,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>2427</v>
+        <v>2426</v>
       </c>
       <c r="C72" t="s">
         <v>2341</v>
@@ -15763,7 +15860,7 @@
         <v>2340</v>
       </c>
       <c r="G72" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
       <c r="H72" t="s">
         <v>2189</v>
@@ -15792,10 +15889,10 @@
         <v>421</v>
       </c>
       <c r="F73" t="s">
-        <v>2428</v>
+        <v>2427</v>
       </c>
       <c r="G73" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H73" t="s">
         <v>2186</v>
@@ -15807,7 +15904,7 @@
         <v>1</v>
       </c>
       <c r="K73" t="s">
-        <v>2429</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
@@ -15827,10 +15924,10 @@
         <v>421</v>
       </c>
       <c r="F74" t="s">
-        <v>2428</v>
+        <v>2427</v>
       </c>
       <c r="G74" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H74" t="s">
         <v>2186</v>
@@ -15842,7 +15939,7 @@
         <v>1</v>
       </c>
       <c r="K74" t="s">
-        <v>2430</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
@@ -15850,7 +15947,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>2431</v>
+        <v>2430</v>
       </c>
       <c r="C75" t="s">
         <v>2347</v>
@@ -15865,7 +15962,7 @@
         <v>949</v>
       </c>
       <c r="G75" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H75" t="s">
         <v>2178</v>
@@ -15877,7 +15974,7 @@
         <v>1</v>
       </c>
       <c r="K75" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
@@ -15885,7 +15982,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>2433</v>
+        <v>2432</v>
       </c>
       <c r="C76" t="s">
         <v>2349</v>
@@ -15900,7 +15997,7 @@
         <v>949</v>
       </c>
       <c r="G76" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H76" t="s">
         <v>2351</v>
@@ -15932,7 +16029,7 @@
         <v>949</v>
       </c>
       <c r="G77" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
       <c r="H77" t="s">
         <v>2189</v>
@@ -15949,7 +16046,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>2434</v>
+        <v>2433</v>
       </c>
       <c r="C78" t="s">
         <v>2354</v>
@@ -15964,7 +16061,7 @@
         <v>949</v>
       </c>
       <c r="G78" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H78" t="s">
         <v>2356</v>
@@ -15981,7 +16078,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>2435</v>
+        <v>2434</v>
       </c>
       <c r="C79" t="s">
         <v>2357</v>
@@ -15996,7 +16093,7 @@
         <v>927</v>
       </c>
       <c r="G79" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H79" t="s">
         <v>2178</v>
@@ -16008,7 +16105,7 @@
         <v>1</v>
       </c>
       <c r="K79" t="s">
-        <v>2436</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
@@ -16016,7 +16113,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>2437</v>
+        <v>2436</v>
       </c>
       <c r="C80" t="s">
         <v>2359</v>
@@ -16031,19 +16128,19 @@
         <v>927</v>
       </c>
       <c r="G80" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H80" t="s">
         <v>2313</v>
       </c>
       <c r="I80" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
       <c r="J80" t="b">
         <v>1</v>
       </c>
       <c r="K80" t="s">
-        <v>2444</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
@@ -16051,7 +16148,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>2438</v>
+        <v>2437</v>
       </c>
       <c r="C81" t="s">
         <v>2361</v>
@@ -16066,7 +16163,7 @@
         <v>927</v>
       </c>
       <c r="G81" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H81" t="s">
         <v>2363</v>
@@ -16083,7 +16180,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>2439</v>
+        <v>2438</v>
       </c>
       <c r="C82" t="s">
         <v>2364</v>
@@ -16098,13 +16195,13 @@
         <v>927</v>
       </c>
       <c r="G82" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
       <c r="H82" t="s">
         <v>2198</v>
       </c>
       <c r="I82" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
       <c r="J82" t="b">
         <v>1</v>
@@ -16115,7 +16212,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>2440</v>
+        <v>2439</v>
       </c>
       <c r="C83" t="s">
         <v>2366</v>
@@ -16130,13 +16227,13 @@
         <v>2368</v>
       </c>
       <c r="G83" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H83" t="s">
         <v>2178</v>
       </c>
       <c r="I83" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J83" t="b">
         <v>1</v>
@@ -16162,13 +16259,13 @@
         <v>2368</v>
       </c>
       <c r="G84" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
       <c r="H84" t="s">
         <v>2218</v>
       </c>
       <c r="I84" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J84" t="b">
         <v>1</v>
@@ -16179,7 +16276,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>2441</v>
+        <v>2440</v>
       </c>
       <c r="C85" t="s">
         <v>2372</v>
@@ -16191,22 +16288,22 @@
         <v>423</v>
       </c>
       <c r="F85" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="G85" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="H85" t="s">
         <v>2227</v>
       </c>
       <c r="I85" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J85" t="b">
         <v>1</v>
       </c>
       <c r="K85" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
@@ -16226,22 +16323,22 @@
         <v>421</v>
       </c>
       <c r="F86" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="G86" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
       <c r="H86" t="s">
         <v>2186</v>
       </c>
       <c r="I86" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J86" t="b">
         <v>1</v>
       </c>
       <c r="K86" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
@@ -16249,13 +16346,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
       <c r="C87" t="s">
+        <v>2464</v>
+      </c>
+      <c r="D87" t="s">
         <v>2465</v>
-      </c>
-      <c r="D87" t="s">
-        <v>2466</v>
       </c>
       <c r="E87" t="s">
         <v>200</v>
@@ -16264,13 +16361,13 @@
         <v>2368</v>
       </c>
       <c r="G87" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H87" t="s">
         <v>2178</v>
       </c>
       <c r="I87" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J87" t="b">
         <v>1</v>
@@ -16281,13 +16378,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
       <c r="C88" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="D88" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
       <c r="E88" t="s">
         <v>200</v>
@@ -16296,13 +16393,13 @@
         <v>2368</v>
       </c>
       <c r="G88" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H88" t="s">
         <v>2178</v>
       </c>
       <c r="I88" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J88" t="b">
         <v>1</v>
@@ -16314,13 +16411,13 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
       <c r="C89" t="s">
+        <v>2466</v>
+      </c>
+      <c r="D89" t="s">
         <v>2467</v>
-      </c>
-      <c r="D89" t="s">
-        <v>2468</v>
       </c>
       <c r="E89" t="s">
         <v>200</v>
@@ -16329,13 +16426,13 @@
         <v>2368</v>
       </c>
       <c r="G89" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="H89" t="s">
         <v>2178</v>
       </c>
       <c r="I89" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="J89" t="b">
         <v>1</v>
@@ -38207,7 +38304,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55941987-30AF-6648-9A85-31A79E0640F5}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
@@ -38216,16 +38313,17 @@
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" customWidth="1"/>
     <col min="6" max="6" width="31.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="62.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="66.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="88.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="88.33203125" customWidth="1"/>
-    <col min="11" max="11" width="53.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.5" customWidth="1"/>
+    <col min="8" max="8" width="62.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="66.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="79.33203125" customWidth="1"/>
+    <col min="11" max="11" width="90.83203125" customWidth="1"/>
+    <col min="12" max="12" width="62.5" customWidth="1"/>
+    <col min="13" max="13" width="74.1640625" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2115</v>
       </c>
@@ -38242,31 +38340,34 @@
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>2378</v>
+        <v>147</v>
       </c>
       <c r="G1" t="s">
+        <v>2479</v>
+      </c>
+      <c r="H1" t="s">
         <v>146</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>2119</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>2120</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>2166</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>2121</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>2122</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>2123</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2151</v>
       </c>
@@ -38279,29 +38380,30 @@
       <c r="D2" t="s">
         <v>2156</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>2377</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>2124</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>2125</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>2126</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>2127</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>2128</v>
       </c>
-      <c r="M2" t="b">
+      <c r="N2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2152</v>
       </c>
@@ -38317,26 +38419,26 @@
       <c r="F3" t="s">
         <v>2160</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>2129</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>2130</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>2131</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>2132</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>2133</v>
       </c>
-      <c r="M3" t="b">
+      <c r="N3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2153</v>
       </c>
@@ -38352,26 +38454,26 @@
       <c r="F4" t="s">
         <v>2161</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>2134</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>2135</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>2136</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>2137</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>2138</v>
       </c>
-      <c r="M4" t="b">
+      <c r="N4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2154</v>
       </c>
@@ -38387,26 +38489,26 @@
       <c r="F5" t="s">
         <v>2162</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>2139</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>2140</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>2141</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>2142</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>2143</v>
       </c>
-      <c r="M5" t="b">
+      <c r="N5" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>2155</v>
       </c>
@@ -38419,29 +38521,30 @@
       <c r="D6" t="s">
         <v>2159</v>
       </c>
+      <c r="E6" s="9"/>
       <c r="F6" t="s">
         <v>2163</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>2144</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>2145</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>2146</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>2147</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>2148</v>
       </c>
-      <c r="M6" t="b">
+      <c r="N6" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2167</v>
       </c>
@@ -38457,34 +38560,76 @@
       <c r="F7" t="s">
         <v>2169</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>2170</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>2173</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>2174</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>2175</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>2171</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" s="8" t="s">
         <v>2172</v>
       </c>
-      <c r="M7" t="b">
+      <c r="N7" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="F8" s="6"/>
+    <row r="8" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>2475</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2165</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2476</v>
+      </c>
+      <c r="E8" s="9">
+        <v>45994</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2477</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>2377</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>2483</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>2482</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>2480</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>2481</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>2478</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>2484</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{DB08D9B6-F3C8-E84F-AFA0-CD1E52770AC7}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{0D225B07-4494-C44D-997D-1695264A8219}"/>
+    <hyperlink ref="G8" r:id="rId2" xr:uid="{F237ABC7-87F1-A443-83D7-225DCF79C51C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -71777,7 +71922,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
@@ -71803,873 +71948,889 @@
       </c>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
-        <v>46227</v>
+        <v>46235</v>
       </c>
       <c r="B2" t="s">
-        <v>2010</v>
+        <v>2473</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>2011</v>
+        <v>2474</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>2009</v>
+        <v>2472</v>
       </c>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B3" t="s">
-        <v>1929</v>
+        <v>2010</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>1928</v>
+        <v>2011</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1930</v>
+        <v>2009</v>
       </c>
       <c r="G3" s="5"/>
     </row>
     <row r="4" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="B4" t="s">
-        <v>1923</v>
+        <v>1929</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>1924</v>
+        <v>1928</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1922</v>
+        <v>1930</v>
       </c>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="B5" t="s">
-        <v>1870</v>
+        <v>1923</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>1872</v>
+        <v>1924</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1871</v>
+        <v>1922</v>
       </c>
       <c r="G5" s="5"/>
     </row>
     <row r="6" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
-        <v>46199</v>
+        <v>46206</v>
       </c>
       <c r="B6" t="s">
-        <v>1751</v>
+        <v>1870</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>1750</v>
+        <v>1872</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1752</v>
+        <v>1871</v>
       </c>
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
-        <v>46192</v>
+        <v>46199</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>1751</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>5</v>
+        <v>1750</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>6</v>
+        <v>1752</v>
       </c>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
-        <v>46185</v>
+        <v>46192</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
-        <v>46171</v>
+        <v>46178</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9">
-        <v>46164</v>
+        <v>46171</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
-        <v>46157</v>
+        <v>46164</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G12" s="5"/>
     </row>
     <row r="13" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
-        <v>46143</v>
+        <v>46150</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
-        <v>46136</v>
+        <v>46143</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
-        <v>46129</v>
+        <v>46136</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G16" s="5"/>
     </row>
     <row r="17" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
-        <v>46115</v>
+        <v>46129</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G17" s="5"/>
     </row>
     <row r="18" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
-        <v>46094</v>
+        <v>46115</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G18" s="5"/>
     </row>
     <row r="19" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
-        <v>46087</v>
+        <v>46094</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
-        <v>46080</v>
+        <v>46087</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G20" s="5"/>
     </row>
     <row r="21" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
-        <v>46073</v>
+        <v>46080</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
-        <v>46066</v>
+        <v>46073</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G22" s="5"/>
     </row>
     <row r="23" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
-        <v>46059</v>
+        <v>46066</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>50</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
-        <v>46052</v>
+        <v>46059</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G24" s="5"/>
     </row>
     <row r="25" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
+        <v>46045</v>
+      </c>
+      <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="5"/>
+    </row>
+    <row r="27" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="9">
         <v>46038</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C27" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="G26" s="5"/>
-    </row>
-    <row r="27" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="9">
-        <v>46031</v>
-      </c>
-      <c r="B27" t="s">
-        <v>62</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="G27" s="5"/>
     </row>
     <row r="28" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
+        <v>46031</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="9">
         <v>46024</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C29" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="G28" s="5"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="9">
-        <v>46017</v>
-      </c>
-      <c r="B29" t="s">
-        <v>68</v>
-      </c>
-      <c r="C29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="G29" s="5"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
+        <v>46017</v>
+      </c>
+      <c r="B30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G30" s="5"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="9">
         <v>46010</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>71</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D31" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="G30" s="5"/>
-    </row>
-    <row r="31" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="9">
-        <v>46003</v>
-      </c>
-      <c r="B31" t="s">
-        <v>74</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="G31" s="5"/>
     </row>
     <row r="32" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
-        <v>45996</v>
+        <v>46003</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="G32" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="G32" s="5"/>
     </row>
     <row r="33" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
-        <v>45989</v>
+        <v>45996</v>
       </c>
       <c r="B33" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
-        <v>45982</v>
+        <v>45989</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
-        <v>45975</v>
+        <v>45982</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G35" s="6"/>
     </row>
     <row r="36" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
-        <v>45968</v>
+        <v>45975</v>
       </c>
       <c r="B36" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G36" s="6"/>
     </row>
     <row r="37" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
+        <v>45968</v>
+      </c>
+      <c r="B37" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="9">
         <v>45961</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C38" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D38" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="9">
+      <c r="G38" s="6"/>
+    </row>
+    <row r="39" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="9">
         <v>45954</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>93</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C39" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D39" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="39" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="9">
+      <c r="G39" s="6"/>
+    </row>
+    <row r="40" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="9">
         <v>45947</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>96</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C40" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D40" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="G39" s="6"/>
-    </row>
-    <row r="40" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="9">
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="9">
         <v>45940</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C41" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D41" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="G40" s="6"/>
-    </row>
-    <row r="41" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="9">
-        <v>45933</v>
-      </c>
-      <c r="B41" t="s">
-        <v>102</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="G41" s="6"/>
     </row>
     <row r="42" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
+        <v>45933</v>
+      </c>
+      <c r="B42" t="s">
+        <v>102</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G42" s="6"/>
+    </row>
+    <row r="43" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="9">
         <v>45926</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>105</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C43" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="43" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="9">
+      <c r="G43" s="6"/>
+    </row>
+    <row r="44" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="9">
         <v>45919</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>108</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C44" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D44" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="9">
-        <v>45912</v>
-      </c>
-      <c r="B44" t="s">
-        <v>111</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="G44" s="6"/>
     </row>
     <row r="45" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
+        <v>45912</v>
+      </c>
+      <c r="B45" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G45" s="6"/>
+    </row>
+    <row r="46" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="9">
         <v>45905</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>114</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C46" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D46" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="9">
+      <c r="G46" s="6"/>
+    </row>
+    <row r="47" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="9">
         <v>45898</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>117</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="C47" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D47" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="9">
+      <c r="G47" s="6"/>
+    </row>
+    <row r="48" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="9">
         <v>45891</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>120</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="C48" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="D48" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="G47" s="6"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="9">
+      <c r="G48" s="6"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="9">
         <v>45884</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>123</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" t="s">
         <v>123</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D49" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="G48" s="6"/>
-    </row>
-    <row r="49" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="9">
-        <v>45877</v>
-      </c>
-      <c r="B49" t="s">
-        <v>125</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9">
+        <v>45877</v>
+      </c>
+      <c r="B50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G50" s="6"/>
+    </row>
+    <row r="51" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="9">
         <v>45870</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B51" t="s">
         <v>128</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C51" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="G50" s="6"/>
-    </row>
-    <row r="51" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="9">
-        <v>45863</v>
-      </c>
-      <c r="B51" t="s">
-        <v>131</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>133</v>
       </c>
       <c r="G51" s="6"/>
     </row>
     <row r="52" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9">
-        <v>45856</v>
+        <v>45863</v>
       </c>
       <c r="B52" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G52" s="6"/>
     </row>
     <row r="53" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="9">
-        <v>45849</v>
+        <v>45856</v>
       </c>
       <c r="B53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="9">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="B54" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G54" s="6"/>
     </row>
     <row r="55" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="9">
+        <v>45842</v>
+      </c>
+      <c r="B55" t="s">
+        <v>140</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G55" s="6"/>
+    </row>
+    <row r="56" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="9">
         <v>45835</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>143</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C56" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="D55" s="6" t="s">
+      <c r="D56" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="G55" s="6"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="C56" s="8"/>
+      <c r="G56" s="6"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C57" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="D8" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="D9" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
-    <hyperlink ref="D10" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
-    <hyperlink ref="D11" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
-    <hyperlink ref="D12" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
-    <hyperlink ref="D13" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
-    <hyperlink ref="D15" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
-    <hyperlink ref="D17" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
-    <hyperlink ref="D18" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
-    <hyperlink ref="D19" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
-    <hyperlink ref="D20" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
-    <hyperlink ref="D21" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
-    <hyperlink ref="D22" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
-    <hyperlink ref="D23" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
-    <hyperlink ref="D24" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
-    <hyperlink ref="D25" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
-    <hyperlink ref="D26" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
-    <hyperlink ref="D27" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
-    <hyperlink ref="D28" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
-    <hyperlink ref="D29" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
-    <hyperlink ref="D30" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
-    <hyperlink ref="D31" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
-    <hyperlink ref="D32" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
-    <hyperlink ref="D33" r:id="rId25" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
-    <hyperlink ref="D34" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
-    <hyperlink ref="D35" r:id="rId27" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
-    <hyperlink ref="D36" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
-    <hyperlink ref="D37" r:id="rId29" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
-    <hyperlink ref="D38" r:id="rId30" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
-    <hyperlink ref="D39" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
-    <hyperlink ref="D40" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
-    <hyperlink ref="D41" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
-    <hyperlink ref="D42" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
-    <hyperlink ref="D43" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
-    <hyperlink ref="D44" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
-    <hyperlink ref="D45" r:id="rId37" xr:uid="{00000000-0004-0000-0400-000024000000}"/>
-    <hyperlink ref="D46" r:id="rId38" xr:uid="{00000000-0004-0000-0400-000025000000}"/>
-    <hyperlink ref="D47" r:id="rId39" xr:uid="{00000000-0004-0000-0400-000026000000}"/>
-    <hyperlink ref="D48" r:id="rId40" xr:uid="{00000000-0004-0000-0400-000027000000}"/>
-    <hyperlink ref="D49" r:id="rId41" xr:uid="{00000000-0004-0000-0400-000028000000}"/>
-    <hyperlink ref="D50" r:id="rId42" xr:uid="{00000000-0004-0000-0400-000029000000}"/>
-    <hyperlink ref="D51" r:id="rId43" xr:uid="{00000000-0004-0000-0400-00002A000000}"/>
-    <hyperlink ref="D52" r:id="rId44" xr:uid="{00000000-0004-0000-0400-00002B000000}"/>
-    <hyperlink ref="D53" r:id="rId45" xr:uid="{00000000-0004-0000-0400-00002C000000}"/>
-    <hyperlink ref="D54" r:id="rId46" xr:uid="{00000000-0004-0000-0400-00002D000000}"/>
-    <hyperlink ref="D55" r:id="rId47" xr:uid="{00000000-0004-0000-0400-00002E000000}"/>
-    <hyperlink ref="D7" r:id="rId48" xr:uid="{F9990143-F9A9-124E-BCC1-1FAB349A9366}"/>
-    <hyperlink ref="D6" r:id="rId49" xr:uid="{EE336F4B-5EFC-034A-9FF6-DB34FC42BBA7}"/>
-    <hyperlink ref="D5" r:id="rId50" xr:uid="{4FE02816-5803-B546-8B3C-00FB300D94B2}"/>
-    <hyperlink ref="D4" r:id="rId51" xr:uid="{8E240BDD-02FF-CA47-B5D9-FD7E9FCA5AEA}"/>
-    <hyperlink ref="D3" r:id="rId52" xr:uid="{77C8CFB5-83B9-D448-AFCE-DD617D9A359D}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="D10" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="D11" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="D12" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="D13" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="D14" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="D16" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="D18" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="D19" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="D20" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="D21" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="D22" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="D24" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="D25" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="D26" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="D27" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
+    <hyperlink ref="D28" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
+    <hyperlink ref="D29" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
+    <hyperlink ref="D30" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
+    <hyperlink ref="D31" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
+    <hyperlink ref="D32" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
+    <hyperlink ref="D33" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
+    <hyperlink ref="D34" r:id="rId25" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
+    <hyperlink ref="D35" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
+    <hyperlink ref="D36" r:id="rId27" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
+    <hyperlink ref="D37" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
+    <hyperlink ref="D38" r:id="rId29" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
+    <hyperlink ref="D39" r:id="rId30" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
+    <hyperlink ref="D40" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
+    <hyperlink ref="D41" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
+    <hyperlink ref="D42" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
+    <hyperlink ref="D43" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
+    <hyperlink ref="D44" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
+    <hyperlink ref="D45" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
+    <hyperlink ref="D46" r:id="rId37" xr:uid="{00000000-0004-0000-0400-000024000000}"/>
+    <hyperlink ref="D47" r:id="rId38" xr:uid="{00000000-0004-0000-0400-000025000000}"/>
+    <hyperlink ref="D48" r:id="rId39" xr:uid="{00000000-0004-0000-0400-000026000000}"/>
+    <hyperlink ref="D49" r:id="rId40" xr:uid="{00000000-0004-0000-0400-000027000000}"/>
+    <hyperlink ref="D50" r:id="rId41" xr:uid="{00000000-0004-0000-0400-000028000000}"/>
+    <hyperlink ref="D51" r:id="rId42" xr:uid="{00000000-0004-0000-0400-000029000000}"/>
+    <hyperlink ref="D52" r:id="rId43" xr:uid="{00000000-0004-0000-0400-00002A000000}"/>
+    <hyperlink ref="D53" r:id="rId44" xr:uid="{00000000-0004-0000-0400-00002B000000}"/>
+    <hyperlink ref="D54" r:id="rId45" xr:uid="{00000000-0004-0000-0400-00002C000000}"/>
+    <hyperlink ref="D55" r:id="rId46" xr:uid="{00000000-0004-0000-0400-00002D000000}"/>
+    <hyperlink ref="D56" r:id="rId47" xr:uid="{00000000-0004-0000-0400-00002E000000}"/>
+    <hyperlink ref="D8" r:id="rId48" xr:uid="{F9990143-F9A9-124E-BCC1-1FAB349A9366}"/>
+    <hyperlink ref="D7" r:id="rId49" xr:uid="{EE336F4B-5EFC-034A-9FF6-DB34FC42BBA7}"/>
+    <hyperlink ref="D6" r:id="rId50" xr:uid="{4FE02816-5803-B546-8B3C-00FB300D94B2}"/>
+    <hyperlink ref="D5" r:id="rId51" xr:uid="{8E240BDD-02FF-CA47-B5D9-FD7E9FCA5AEA}"/>
+    <hyperlink ref="D4" r:id="rId52" xr:uid="{77C8CFB5-83B9-D448-AFCE-DD617D9A359D}"/>
+    <hyperlink ref="D3" r:id="rId53" xr:uid="{7282EB94-FBFF-C64E-9C65-3E4E1C662EA7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
CookwithTK fixed canvas and ingredients size
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekookuniverse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B21960F-97BE-B24E-A495-749B2C98A570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D36BB71-EB88-0542-B649-3BC56707B32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-33320" yWindow="2920" windowWidth="29560" windowHeight="19060" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3959" uniqueCount="2498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3959" uniqueCount="2497">
   <si>
     <t>date</t>
   </si>
@@ -13239,9 +13239,6 @@
 Grate Parmigiano Reggiano into the pasta and continue cooking briefly.
 Turn off the heat and serve.
 Top with additional grated Parmigiano Reggiano and freshly ground pepper.</t>
-  </si>
-  <si>
-    <t>Shrimp Pasta</t>
   </si>
 </sst>
 </file>
@@ -38960,7 +38957,7 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>2497</v>
+        <v>2153</v>
       </c>
       <c r="B10" t="s">
         <v>2165</v>
@@ -38970,6 +38967,9 @@
       </c>
       <c r="E10" s="9">
         <v>45985</v>
+      </c>
+      <c r="O10" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>